<commit_message>
Wire PSM+biz persona into agents; add Analyst Questions + AI Thoughts tabs (I-075, I-076)
- estimate_writer.txt: FL PSM 20yr expert + business/sales pro — knows flood zones, B2B tone, estimate-as-conversion-doc
- estimate_reviewer.txt: domain sanity checks added (ALTA floor, EC for flood zones, Boundary ceiling)
- Historical_Analysis_Report.xlsx: 2 new tabs — 'Analyst Questions' (13 biz/finance/sales Qs with data answers) + 'AI Thoughts - Today' (live invoicing reasoning for May 28 scenario)
- issues/issue.md: log I-075 (no domain persona) + I-076 (report missing AI perspective tabs)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Historical_Analysis_Report.xlsx
+++ b/Historical_Analysis_Report.xlsx
@@ -16,6 +16,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AR Analysis" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Commercial vs Residential" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI Action Items" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Analyst Questions" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI Thoughts - Today" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -25,7 +27,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="25">
+  <fonts count="27">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -170,6 +172,18 @@
       <color rgb="002E75B6"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="002D6A2D"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FF4B4B"/>
+      <sz val="10"/>
+    </font>
   </fonts>
   <fills count="18">
     <fill>
@@ -285,7 +299,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="86">
+  <cellXfs count="91">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -541,6 +555,21 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1104,7 +1133,7 @@
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Source: nexgen_ftf_db (AWS RDS production)  |  Generated: May 27, 2026</t>
+          <t>Source: nexgen_ftf_db (AWS RDS production)  |  Generated: May 28, 2026</t>
         </is>
       </c>
     </row>
@@ -1509,6 +1538,996 @@
     <mergeCell ref="C21:F21"/>
     <mergeCell ref="A13:B13"/>
     <mergeCell ref="C13:D13"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="46" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="3" max="3"/>
+    <col width="36" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="19" t="inlineStr">
+        <is>
+          <t>AI Analyst Questions — Business, Sales &amp; Finance Intelligence</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="36" customHeight="1">
+      <c r="A2" s="80" t="inlineStr">
+        <is>
+          <t>I am your AI business analyst. I have read 2 years of NexGen invoices (47,825 records, $25.6M). Before I can help you run the business better, I need answers to the questions below. Where I already have the data, I've answered it myself. Where data is missing, I flag it for you.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="20" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B3" s="20" t="inlineStr">
+        <is>
+          <t>My Question</t>
+        </is>
+      </c>
+      <c r="C3" s="20" t="inlineStr">
+        <is>
+          <t>What the Data Says</t>
+        </is>
+      </c>
+      <c r="D3" s="20" t="inlineStr">
+        <is>
+          <t>What I Need / Action</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="36" t="inlineStr">
+        <is>
+          <t>REVENUE REALITY — Potential vs Actual</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="72" customHeight="1">
+      <c r="A5" s="20" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B5" s="21" t="inlineStr">
+        <is>
+          <t>What is the difference between your order revenue numbers and your actual business revenue?</t>
+        </is>
+      </c>
+      <c r="C5" s="23" t="inlineStr">
+        <is>
+          <t>Yr2: $13.2M INVOICED (potential). Only ~$6.65M actually collected (paid). $6.57M is still outstanding — 49.7% of revenue is uncollected. Every time someone says '$13M revenue' they are quoting POTENTIAL, not cash.</t>
+        </is>
+      </c>
+      <c r="D5" s="32" t="inlineStr">
+        <is>
+          <t>Confirm: does the team track COLLECTED revenue separately? Jessica's AR agent should report both numbers on every digest.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="72" customHeight="1">
+      <c r="A6" s="20" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B6" s="17" t="inlineStr">
+        <is>
+          <t>How much revenue is locked in 'Quote' orders that were never converted?</t>
+        </is>
+      </c>
+      <c r="C6" s="85" t="inlineStr">
+        <is>
+          <t>Yr2: 1,721 Quote orders at avg $926 = $1.59M in potential revenue sitting unclassified. Yr1 had 3,379 Quotes at avg $853 = $2.88M. If even 40% of Yr2 Quotes were converted and paid = $636K additional revenue.</t>
+        </is>
+      </c>
+      <c r="D6" s="32" t="inlineStr">
+        <is>
+          <t>What is the actual Quote-to-Paid conversion rate? I need: how many Quote orders eventually became Delivered/Complete. This is the single most valuable number for sales planning.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="72" customHeight="1">
+      <c r="A7" s="20" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B7" s="21" t="inlineStr">
+        <is>
+          <t>How much revenue was lost to canceled orders?</t>
+        </is>
+      </c>
+      <c r="C7" s="23" t="inlineStr">
+        <is>
+          <t>I can see partial cancellation billing in the data ('Cancel after office prep 10%', 'Cancel after field work 50%') but I do not have total cancellation counts or lost revenue. These show up as informal service types — they are NOT in the canonical catalogue.</t>
+        </is>
+      </c>
+      <c r="D7" s="32" t="inlineStr">
+        <is>
+          <t>Pull all orders with status=Cancelled from FTF API. How many? What service types? What was the original quote? Cancel rate and lost revenue are metrics the team should review monthly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="36" t="inlineStr">
+        <is>
+          <t>QUOTE PIPELINE — Where Does Revenue Die?</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="72" customHeight="1">
+      <c r="A9" s="20" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B9" s="17" t="inlineStr">
+        <is>
+          <t>What happens to a Quote order after it arrives? What are the drop-off points?</t>
+        </is>
+      </c>
+      <c r="C9" s="85" t="inlineStr">
+        <is>
+          <t>Current pipeline: Quote arrives -&gt; Classifier flags it -&gt; Human Gate -&gt; awaiting approval. If human does not approve within 24h, escalation to Ryan/Wyatt. But I do NOT know: how many Quotes expire (60-day auto-cancel per FTF portal)? How many are rejected vs converted?</t>
+        </is>
+      </c>
+      <c r="D9" s="32" t="inlineStr">
+        <is>
+          <t>I need a funnel report: Quotes received -&gt; Classified -&gt; Approved -&gt; Sent -&gt; Paid. Each stage where orders drop off = lost revenue opportunity. BUILD: Quote pipeline funnel as a monthly KPI.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="72" customHeight="1">
+      <c r="A10" s="20" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B10" s="21" t="inlineStr">
+        <is>
+          <t>Why did Quote volume drop 49% from Yr1 to Yr2 (3,379 -&gt; 1,721)?</t>
+        </is>
+      </c>
+      <c r="C10" s="23" t="inlineStr">
+        <is>
+          <t>Two possible explanations: (A) FTF staff are classifying orders faster so fewer arrive as Quote, or (B) overall new-order intake dropped 49%. Revenue grew +6.5% despite this drop — so explanation A is more likely (better classification, same or higher quality orders).</t>
+        </is>
+      </c>
+      <c r="D10" s="32" t="inlineStr">
+        <is>
+          <t>Confirm with Robert: is the team entering service types more carefully in Yr2? If yes, this is a positive data quality improvement. If no, new-order intake may have actually declined — which is a sales problem.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="36" t="inlineStr">
+        <is>
+          <t>AR RISK — $6.57M Uncollected</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="72" customHeight="1">
+      <c r="A12" s="20" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B12" s="17" t="inlineStr">
+        <is>
+          <t>Which clients owe the most money? Are the largest AR balances B2B or individual?</t>
+        </is>
+      </c>
+      <c r="C12" s="85" t="inlineStr">
+        <is>
+          <t>I know: 49.7% of Yr2 revenue ($6.57M) is unpaid. 8,212 invoices unpaid. Avg unpaid invoice = $799. But I do NOT have: a client-level AR aging breakdown. B2B clients (title companies, builders) tend to have larger balances.</t>
+        </is>
+      </c>
+      <c r="D12" s="32" t="inlineStr">
+        <is>
+          <t>Jessica needs: a top-50 AR aging report by client, sorted by total owed. This is the #1 collection priority. If even the top 10 clients pay, that could be $500K-$1M recovered.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="72" customHeight="1">
+      <c r="A13" s="20" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B13" s="21" t="inlineStr">
+        <is>
+          <t>Are invoices getting paid faster or slower year over year?</t>
+        </is>
+      </c>
+      <c r="C13" s="23" t="inlineStr">
+        <is>
+          <t>Payment volume shifted: check payments -31% (15K-&gt;10K), CC payments +71% (2.6K-&gt;4.5K). CC payments are typically faster (same-day authorization vs check clearing). BUT: unpaid invoices grew +21% despite more CC volume — suggesting more invoices are never paid at all (not just slow payers).</t>
+        </is>
+      </c>
+      <c r="D13" s="32" t="inlineStr">
+        <is>
+          <t>Track: avg days-to-payment by payment type. If CC avg = 2 days and check avg = 30 days, push CC in all estimate emails. Also: how many invoices have been unpaid &gt;90 days? &gt;180 days? &gt;1 year?</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="A14" s="36" t="inlineStr">
+        <is>
+          <t>GROWTH OPPORTUNITIES — Where Is the Money?</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="72" customHeight="1">
+      <c r="A15" s="20" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B15" s="17" t="inlineStr">
+        <is>
+          <t>Commercial is 2.8% of volume but 10.5% of revenue. Are we maximizing commercial?</t>
+        </is>
+      </c>
+      <c r="C15" s="85" t="inlineStr">
+        <is>
+          <t>Yr2: 642 commercial orders, avg $2,159. If NexGen could add 100 more commercial jobs at $2,159 avg = $215,900 additional revenue. Commercial multiplier grew from 3.1x to 4.1x — NexGen is pricing commercial work correctly now.</t>
+        </is>
+      </c>
+      <c r="D15" s="32" t="inlineStr">
+        <is>
+          <t>How many commercial quotes are being rejected or expiring? Commercial pipeline needs priority handling. Every lost commercial job = 4 lost residential jobs in revenue value.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="72" customHeight="1">
+      <c r="A16" s="20" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B16" s="21" t="inlineStr">
+        <is>
+          <t>Panhandle counties averaged $1,720-$2,466 per job in Yr1. Why did they disappear in Yr2?</t>
+        </is>
+      </c>
+      <c r="C16" s="23" t="inlineStr">
+        <is>
+          <t>Santa Rosa ($2,466 avg), Escambia ($2,210), Bay ($2,000), Leon ($1,720) — all appeared in Yr1, ZERO orders in Yr2. Combined Yr1 Panhandle revenue: ~$165K from 85 orders (avg ~$1,940). If these counties are no longer being served, that is $165K/year lost.</t>
+        </is>
+      </c>
+      <c r="D16" s="32" t="inlineStr">
+        <is>
+          <t>Bobby/Robert: are we still taking Panhandle jobs? If crew coverage is the issue, can we use contract surveyors? These are the highest-priced jobs in the state — worth solving.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="72" customHeight="1">
+      <c r="A17" s="20" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B17" s="17" t="inlineStr">
+        <is>
+          <t>Spot Survey surged from 10 to 106 orders (+960%). What is driving this?</t>
+        </is>
+      </c>
+      <c r="C17" s="85" t="inlineStr">
+        <is>
+          <t>Spot Survey (New Client) = Foundation Tie-In in canonical terms. Avg price $589. 106 orders x $589 = $62K in Yr2. This surge suggests either a new client vertical or more new clients being onboarded needing foundation surveys before construction.</t>
+        </is>
+      </c>
+      <c r="D17" s="32" t="inlineStr">
+        <is>
+          <t>Who are the new Spot Survey clients? Is this from one builder/developer relationship? If one client is driving 100 jobs, that is a strategic relationship to protect. If it is many new clients, what marketing channel brought them in?</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="36" t="inlineStr">
+        <is>
+          <t>OPERATIONAL GAPS — What I Cannot See But Need To</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="72" customHeight="1">
+      <c r="A19" s="20" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="B19" s="21" t="inlineStr">
+        <is>
+          <t>What is NexGen's actual cash position month-to-month? I only see invoiced amounts.</t>
+        </is>
+      </c>
+      <c r="C19" s="23" t="inlineStr">
+        <is>
+          <t>I can see what was billed ($13.2M) and what is unpaid ($6.57M). But I cannot see: when payments cleared, what were operating costs, payroll, or net profit. The $6.65M collected is gross — not net.</t>
+        </is>
+      </c>
+      <c r="D19" s="32" t="inlineStr">
+        <is>
+          <t>For real financial health monitoring, AI needs access to QuickBooks or the actual cash accounts. The FTF Books data I have is accounts receivable only. Jessica or Ryan: can QuickBooks data be connected?</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="72" customHeight="1">
+      <c r="A20" s="20" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="B20" s="17" t="inlineStr">
+        <is>
+          <t>B-II Title Review billed 11 times in Yr1 and ZERO in Yr2. What happened?</t>
+        </is>
+      </c>
+      <c r="C20" s="85" t="inlineStr">
+        <is>
+          <t>B-II Title Review ($450 catalogue price) completely disappeared from Yr2 billing. Either: (A) NexGen stopped offering it, (B) it is being billed under another name, or (C) those clients went elsewhere. Also conflicts with I-055 (auto-quote vs flag debate).</t>
+        </is>
+      </c>
+      <c r="D20" s="32" t="inlineStr">
+        <is>
+          <t>Robert must confirm: is B-II Title Review still offered? If yes, why is it not appearing? If no, remove from catalogue. This is an unanswered question that has been open since I-055 (2026-05-26).</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="72" customHeight="1">
+      <c r="A21" s="20" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="B21" s="21" t="inlineStr">
+        <is>
+          <t>Are seasonal staffing levels matched to the March-April peak?</t>
+        </is>
+      </c>
+      <c r="C21" s="23" t="inlineStr">
+        <is>
+          <t>March-April 2026 = busiest months: 2,219 and 2,212 orders respectively. Nov 2025 = slowest at 1,564 orders. Peak/trough ratio = 1.42x. If crew size is fixed, March-April will have backlogs and customer delays.</t>
+        </is>
+      </c>
+      <c r="D21" s="32" t="inlineStr">
+        <is>
+          <t>Bobby: what is current crew headcount? Do we add contract surveyors in March-April? Weather monitoring agent (I-070) should alert on peak months + bad weather together — that combination is highest delay risk.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A18:D18"/>
+    <mergeCell ref="A8:D8"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A11:D11"/>
+    <mergeCell ref="A14:D14"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="38" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="19" t="inlineStr">
+        <is>
+          <t>AI Thoughts — What Would I Do If I Had to Invoice Today's Jobs?</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="36" customHeight="1">
+      <c r="A2" s="80" t="inlineStr">
+        <is>
+          <t>TODAY: 2026-05-28 (Wednesday, May). Based on May 2026 actuals (~80 orders/day, avg $556), here is exactly what I would do — service by service — if those orders arrived right now. I am thinking as a FL PSM expert + business analyst. This is my live reasoning.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="24" customHeight="1">
+      <c r="A3" s="86" t="inlineStr">
+        <is>
+          <t>SECTION 1 — Expected Order Mix Today (Based on May 2026 Actuals)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="36" t="inlineStr">
+        <is>
+          <t>Service Type</t>
+        </is>
+      </c>
+      <c r="B4" s="36" t="inlineStr">
+        <is>
+          <t>Expected Today</t>
+        </is>
+      </c>
+      <c r="C4" s="36" t="inlineStr">
+        <is>
+          <t>Avg Price</t>
+        </is>
+      </c>
+      <c r="D4" s="36" t="inlineStr">
+        <is>
+          <t>Auto-Quote?</t>
+        </is>
+      </c>
+      <c r="E4" s="36" t="inlineStr">
+        <is>
+          <t>Est. Revenue</t>
+        </is>
+      </c>
+      <c r="F4" s="36" t="inlineStr">
+        <is>
+          <t>My Reasoning</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="72" customHeight="1">
+      <c r="A5" s="24" t="inlineStr">
+        <is>
+          <t>Boundary Survey
+(Land Survey Only / Land Survey &amp; Elevation)</t>
+        </is>
+      </c>
+      <c r="B5" s="25" t="inlineStr">
+        <is>
+          <t>~46 orders</t>
+        </is>
+      </c>
+      <c r="C5" s="25" t="inlineStr">
+        <is>
+          <t>$556</t>
+        </is>
+      </c>
+      <c r="D5" s="87" t="inlineStr">
+        <is>
+          <t>YES — if county known, no VE zone</t>
+        </is>
+      </c>
+      <c r="E5" s="45" t="inlineStr">
+        <is>
+          <t>~$25,600</t>
+        </is>
+      </c>
+      <c r="F5" s="26" t="inlineStr">
+        <is>
+          <t>The dominant service at 57% of volume. I use county-based pricing: Palm Beach $572, Broward $512, Hillsborough $575. If flood zone = AE, I add Elevation Certificate ($225). If county is MISSING, I flag for human — cannot price without it. If flood zone = VE, I flag regardless of service type.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="72" customHeight="1">
+      <c r="A6" s="27" t="inlineStr">
+        <is>
+          <t>Quote (Unclassified orders from FTF)</t>
+        </is>
+      </c>
+      <c r="B6" s="28" t="inlineStr">
+        <is>
+          <t>~6 orders</t>
+        </is>
+      </c>
+      <c r="C6" s="28" t="inlineStr">
+        <is>
+          <t>$926 avg</t>
+        </is>
+      </c>
+      <c r="D6" s="88" t="inlineStr">
+        <is>
+          <t>NO — always flag</t>
+        </is>
+      </c>
+      <c r="E6" s="61" t="inlineStr">
+        <is>
+          <t>$0 auto-quoted
+$5,556 potential</t>
+        </is>
+      </c>
+      <c r="F6" s="29" t="inlineStr">
+        <is>
+          <t>These arrive with service_type='Quote' — FTF staff did not classify them yet. My classifier cannot guess what survey is needed. Average value is HIGH ($926) — these are likely complex or commercial. I send all 6 to human gate immediately with flag: 'service_type=Quote — unclassified by FTF staff.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="72" customHeight="1">
+      <c r="A7" s="24" t="inlineStr">
+        <is>
+          <t>Elevation Certificate (standalone)</t>
+        </is>
+      </c>
+      <c r="B7" s="25" t="inlineStr">
+        <is>
+          <t>~2 orders</t>
+        </is>
+      </c>
+      <c r="C7" s="25" t="inlineStr">
+        <is>
+          <t>$271</t>
+        </is>
+      </c>
+      <c r="D7" s="87" t="inlineStr">
+        <is>
+          <t>YES — if individual, no VE zone</t>
+        </is>
+      </c>
+      <c r="E7" s="45" t="inlineStr">
+        <is>
+          <t>~$540</t>
+        </is>
+      </c>
+      <c r="F7" s="26" t="inlineStr">
+        <is>
+          <t>These are simpler standalone certs. I check: is it AE zone (standard EC) or VE zone (flag for specialist)? Individual client + AE zone = auto-quote $271. Commercial or VE = flag. I note on the estimate: FEMA flood zone designation, why the EC is needed, and that NexGen is a licensed FL PSM.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="72" customHeight="1">
+      <c r="A8" s="27" t="inlineStr">
+        <is>
+          <t>ALTA Table A Survey</t>
+        </is>
+      </c>
+      <c r="B8" s="28" t="inlineStr">
+        <is>
+          <t>~1 order</t>
+        </is>
+      </c>
+      <c r="C8" s="28" t="inlineStr">
+        <is>
+          <t>$5,075 avg</t>
+        </is>
+      </c>
+      <c r="D8" s="88" t="inlineStr">
+        <is>
+          <t>NO — always flag</t>
+        </is>
+      </c>
+      <c r="E8" s="61" t="inlineStr">
+        <is>
+          <t>$0 auto-quoted
+$5,075 potential</t>
+        </is>
+      </c>
+      <c r="F8" s="29" t="inlineStr">
+        <is>
+          <t>ALTA is always human review. No exceptions. Avg Yr2 price is $5,075 but every ALTA is custom-scoped. I cannot auto-quote without knowing: table A items requested, acreage, encumbrances, title commitment. I flag immediately: 'ALTA — custom scope required, Bobby/Robert must review.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="72" customHeight="1">
+      <c r="A9" s="24" t="inlineStr">
+        <is>
+          <t>Update Survey / Re-Survey</t>
+        </is>
+      </c>
+      <c r="B9" s="25" t="inlineStr">
+        <is>
+          <t>~2 orders</t>
+        </is>
+      </c>
+      <c r="C9" s="25" t="inlineStr">
+        <is>
+          <t>$398</t>
+        </is>
+      </c>
+      <c r="D9" s="87" t="inlineStr">
+        <is>
+          <t>YES — if prior survey on file</t>
+        </is>
+      </c>
+      <c r="E9" s="45" t="inlineStr">
+        <is>
+          <t>~$796</t>
+        </is>
+      </c>
+      <c r="F9" s="26" t="inlineStr">
+        <is>
+          <t>Update surveys recertify a prior NexGen survey. I check: is there a prior survey on file? If yes, price at $398 (Yr2 avg). If this is a competitor's prior survey, I flag — we may need to do a full boundary instead. Important: recertification is 40-60% less cost than a new survey — I make sure this is reflected in the estimate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="72" customHeight="1">
+      <c r="A10" s="27" t="inlineStr">
+        <is>
+          <t>Commercial / B2B (any service type)</t>
+        </is>
+      </c>
+      <c r="B10" s="28" t="inlineStr">
+        <is>
+          <t>~2 orders</t>
+        </is>
+      </c>
+      <c r="C10" s="28" t="inlineStr">
+        <is>
+          <t>$2,159 avg</t>
+        </is>
+      </c>
+      <c r="D10" s="88" t="inlineStr">
+        <is>
+          <t>NO — always flag</t>
+        </is>
+      </c>
+      <c r="E10" s="61" t="inlineStr">
+        <is>
+          <t>$0 auto-quoted
+$4,318 potential</t>
+        </is>
+      </c>
+      <c r="F10" s="29" t="inlineStr">
+        <is>
+          <t>Commercial multiplier is 4.1x residential in Yr2. I flag ALL commercial orders for Bobby/Robert. I do not auto-quote commercial even for simple services — complexity factors (walls, pools, drainage, site access) are not captured in the order form and can double the price. Human judgment is required.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="72" customHeight="1">
+      <c r="A11" s="27" t="inlineStr">
+        <is>
+          <t>Monroe County (any service)</t>
+        </is>
+      </c>
+      <c r="B11" s="28" t="inlineStr">
+        <is>
+          <t>~0-1 orders</t>
+        </is>
+      </c>
+      <c r="C11" s="28" t="inlineStr">
+        <is>
+          <t>$1,735 avg</t>
+        </is>
+      </c>
+      <c r="D11" s="88" t="inlineStr">
+        <is>
+          <t>NO — always flag</t>
+        </is>
+      </c>
+      <c r="E11" s="61" t="inlineStr">
+        <is>
+          <t>$0 auto-quoted</t>
+        </is>
+      </c>
+      <c r="F11" s="29" t="inlineStr">
+        <is>
+          <t>Monroe County = Florida Keys. Non-standard pricing due to island access, tidal flood complexity, and CCCL (Coastal Construction Control Line) regulations. I flag every Monroe County order regardless of service type with: 'Monroe County — non-standard pricing, human review required.' This is a hard rule from the classifier.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="24" customHeight="1">
+      <c r="A13" s="86" t="inlineStr">
+        <is>
+          <t>SECTION 2 — My End-of-Day Summary (If I Run the Pipeline Today)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="36" t="inlineStr">
+        <is>
+          <t>Outcome</t>
+        </is>
+      </c>
+      <c r="B14" s="36" t="inlineStr">
+        <is>
+          <t>Count</t>
+        </is>
+      </c>
+      <c r="C14" s="36" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="D14" s="36" t="inlineStr"/>
+      <c r="E14" s="36" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="F14" s="36" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="36" customHeight="1">
+      <c r="A15" s="24" t="inlineStr">
+        <is>
+          <t>Auto-quoted &amp; sent to clients</t>
+        </is>
+      </c>
+      <c r="B15" s="25" t="inlineStr">
+        <is>
+          <t>~50</t>
+        </is>
+      </c>
+      <c r="C15" s="45" t="inlineStr">
+        <is>
+          <t>~$26,936</t>
+        </is>
+      </c>
+      <c r="D15" s="37" t="inlineStr"/>
+      <c r="E15" s="45" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F15" s="26" t="inlineStr">
+        <is>
+          <t>Boundary surveys, ECs, update surveys in known counties. Estimates sent 8 AM-6 PM ET only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="36" customHeight="1">
+      <c r="A16" s="30" t="inlineStr">
+        <is>
+          <t>Flagged — sent to human gate (Bobby/Robert)</t>
+        </is>
+      </c>
+      <c r="B16" s="31" t="inlineStr">
+        <is>
+          <t>~12</t>
+        </is>
+      </c>
+      <c r="C16" s="44" t="inlineStr">
+        <is>
+          <t>$0 (held)</t>
+        </is>
+      </c>
+      <c r="D16" s="40" t="inlineStr"/>
+      <c r="E16" s="44" t="inlineStr">
+        <is>
+          <t>PENDING HUMAN</t>
+        </is>
+      </c>
+      <c r="F16" s="32" t="inlineStr">
+        <is>
+          <t>Quotes, ALTA, commercial, Monroe County, VE zones. Batch digest sent every hour per I-064.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="36" customHeight="1">
+      <c r="A17" s="27" t="inlineStr">
+        <is>
+          <t>Refund requests intercepted</t>
+        </is>
+      </c>
+      <c r="B17" s="28" t="inlineStr">
+        <is>
+          <t>0 expected</t>
+        </is>
+      </c>
+      <c r="C17" s="61" t="inlineStr">
+        <is>
+          <t>$0</t>
+        </is>
+      </c>
+      <c r="D17" s="38" t="inlineStr"/>
+      <c r="E17" s="61" t="inlineStr">
+        <is>
+          <t>JESSICA ONLY</t>
+        </is>
+      </c>
+      <c r="F17" s="29" t="inlineStr">
+        <is>
+          <t>Hard rule (I-063): any refund mentioned in email or order notes -&gt; Jessica immediately. AI never touches.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="36" customHeight="1">
+      <c r="A18" s="17" t="inlineStr">
+        <is>
+          <t>Estimate emails queued (outside hours)</t>
+        </is>
+      </c>
+      <c r="B18" s="48" t="inlineStr">
+        <is>
+          <t>~3</t>
+        </is>
+      </c>
+      <c r="C18" s="89" t="inlineStr">
+        <is>
+          <t>~$1,680</t>
+        </is>
+      </c>
+      <c r="D18" s="47" t="inlineStr"/>
+      <c r="E18" s="89" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="F18" s="85" t="inlineStr">
+        <is>
+          <t>Orders received after 6 PM ET. Will send tomorrow 8 AM. No sends outside business hours.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="22" customHeight="1">
+      <c r="A21" s="67" t="inlineStr">
+        <is>
+          <t>SECTION 3 — What I Still Need to Invoice Better (Knowledge Gaps)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="81" t="inlineStr">
+        <is>
+          <t>Gap</t>
+        </is>
+      </c>
+      <c r="B22" s="81" t="inlineStr">
+        <is>
+          <t>Impact</t>
+        </is>
+      </c>
+      <c r="C22" s="81" t="inlineStr">
+        <is>
+          <t>Who Resolves</t>
+        </is>
+      </c>
+      <c r="D22" s="81" t="inlineStr"/>
+      <c r="E22" s="81" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="F22" s="81" t="inlineStr">
+        <is>
+          <t>Detail</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="54" customHeight="1">
+      <c r="A23" s="27" t="inlineStr">
+        <is>
+          <t>Property complexity data not in order form</t>
+        </is>
+      </c>
+      <c r="B23" s="29" t="inlineStr">
+        <is>
+          <t>I cannot price pools, sheds, wall count, driveways, or lot shape — all major price factors per Ryan's call</t>
+        </is>
+      </c>
+      <c r="C23" s="28" t="inlineStr">
+        <is>
+          <t>Robert / FTF developer</t>
+        </is>
+      </c>
+      <c r="D23" s="38" t="inlineStr"/>
+      <c r="E23" s="66" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="F23" s="29" t="inlineStr">
+        <is>
+          <t>Ryan: 'Same half-acre with pool, 3 walls, shed = $700. Plain house = $350.' Until FTF order form captures complexity, I use county averages only. I may under-quote complex jobs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="54" customHeight="1">
+      <c r="A24" s="30" t="inlineStr">
+        <is>
+          <t>Quote-to-paid conversion rate unknown</t>
+        </is>
+      </c>
+      <c r="B24" s="32" t="inlineStr">
+        <is>
+          <t>I cannot optimize the quote pipeline without knowing how many Quotes convert</t>
+        </is>
+      </c>
+      <c r="C24" s="31" t="inlineStr">
+        <is>
+          <t>Jessica / FTF data pull</t>
+        </is>
+      </c>
+      <c r="D24" s="40" t="inlineStr"/>
+      <c r="E24" s="66" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="F24" s="32" t="inlineStr">
+        <is>
+          <t>If 1,721 Yr2 Quotes have 40% conversion = $636K recovered. If 20% = $318K. This one number changes the AR strategy completely.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="54" customHeight="1">
+      <c r="A25" s="27" t="inlineStr">
+        <is>
+          <t>Crew location / schedule not available to me</t>
+        </is>
+      </c>
+      <c r="B25" s="29" t="inlineStr">
+        <is>
+          <t>I cannot factor travel cost into pricing for remote counties</t>
+        </is>
+      </c>
+      <c r="C25" s="28" t="inlineStr">
+        <is>
+          <t>Bobby / FieldPack</t>
+        </is>
+      </c>
+      <c r="D25" s="38" t="inlineStr"/>
+      <c r="E25" s="90" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="F25" s="29" t="inlineStr">
+        <is>
+          <t>Ryan: 'Far from crew = charge more.' I have no access to crew schedule. Near-term: add county-based distance tier to pricing (Panhandle = always high, Central FL = baseline).</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="54" customHeight="1">
+      <c r="A26" s="30" t="inlineStr">
+        <is>
+          <t>Florida PSM standards wired in but not tested on real disputes</t>
+        </is>
+      </c>
+      <c r="B26" s="32" t="inlineStr">
+        <is>
+          <t>My FL PSM persona was built from regulations — not from NexGen's actual field decisions</t>
+        </is>
+      </c>
+      <c r="C26" s="31" t="inlineStr">
+        <is>
+          <t>Robert / Mark</t>
+        </is>
+      </c>
+      <c r="D26" s="40" t="inlineStr"/>
+      <c r="E26" s="90" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="F26" s="32" t="inlineStr">
+        <is>
+          <t>Feed me 5-10 real NexGen estimate examples that were disputed or revised. I will learn the gap between the FL standard and what NexGen actually does in the field.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A13:F13"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A3:F3"/>
+    <mergeCell ref="A21:F21"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix invoiced vs collected revenue confusion + log I-077/I-078 (Ryan feedback)
Ryan: 'agent viewing every order as revenue not paid orders — just a data pull'

- Historical_Analysis_Report.xlsx: invoiced ($13.2M) now separated from collected ($6.64M) in
  all KPI cards, AR Analysis tab, Cover insights, and both new tabs
- Cover: red warning banner; 'Collected (Cash In)' KPI card shows YoY -7.8% (cash falling)
- AR Analysis: INVOICED vs COLLECTED distinction prominent; new 'collected dropped' insight
- Analyst Questions + AI Thoughts: both open with Ryan's exact feedback + corrected framing
- issues/issue.md: I-077 CLOSED (terminology fix); I-078 OPEN (real AI analyst agent — future sprint)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Historical_Analysis_Report.xlsx
+++ b/Historical_Analysis_Report.xlsx
@@ -27,7 +27,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="27">
+  <fonts count="26">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -48,8 +48,9 @@
     </font>
     <font>
       <name val="Calibri"/>
+      <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="11"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -67,18 +68,6 @@
       <b val="1"/>
       <color rgb="00000000"/>
       <sz val="13"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="0070AD47"/>
-      <sz val="13"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="0070AD47"/>
-      <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -107,6 +96,18 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
+      <color rgb="0070AD47"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="0070AD47"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="12"/>
     </font>
@@ -126,12 +127,6 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="13"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="10"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -204,12 +199,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="0000B0A0"/>
+        <fgColor rgb="00FF4B4B"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="0070AD47"/>
+        <fgColor rgb="00FFC000"/>
       </patternFill>
     </fill>
     <fill>
@@ -224,27 +219,22 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E2EFDA"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFC000"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FF4B4B"/>
+        <fgColor rgb="00FFE0E0"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFE0E0"/>
+        <fgColor rgb="0070AD47"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
     <fill>
@@ -255,6 +245,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00D9F2EF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0000B0A0"/>
       </patternFill>
     </fill>
     <fill>
@@ -299,7 +294,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="91">
+  <cellXfs count="92">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -313,7 +308,10 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -328,19 +326,16 @@
     <xf numFmtId="0" fontId="9" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -361,6 +356,42 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -370,187 +401,154 @@
     <xf numFmtId="0" fontId="5" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="20" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="19" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="20" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="23" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="23" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="23" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -559,16 +557,16 @@
     <xf numFmtId="0" fontId="16" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="24" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="25" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1133,201 +1131,201 @@
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Source: nexgen_ftf_db (AWS RDS production)  |  Generated: May 28, 2026</t>
+          <t>Source: nexgen_ftf_db (AWS RDS production)  |  Generated: May 28, 2026  |  NOTE: 'Invoiced' = what NexGen billed. 'Collected' = actual cash received (invoiced minus AR). These are NOT the same number.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>Total Revenue</t>
+          <t>Invoiced (Billed)</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>Invoices</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>Avg Price</t>
+          <t>Collected (Cash In)</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>Avg Invoice Price</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="A6" s="7" t="inlineStr">
         <is>
           <t>May 2024 – May</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr">
         <is>
           <t>May 2025 – May</t>
         </is>
       </c>
-      <c r="C6" s="6" t="inlineStr">
+      <c r="C6" s="7" t="inlineStr">
         <is>
           <t>May 2024 – May</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="D6" s="7" t="inlineStr">
         <is>
           <t>May 2025 – May</t>
         </is>
       </c>
-      <c r="E6" s="6" t="inlineStr">
+      <c r="E6" s="7" t="inlineStr">
         <is>
           <t>May 2024 – May</t>
         </is>
       </c>
-      <c r="F6" s="6" t="inlineStr">
+      <c r="F6" s="7" t="inlineStr">
         <is>
           <t>May 2025 – May</t>
         </is>
       </c>
     </row>
     <row r="7" ht="28" customHeight="1">
-      <c r="A7" s="7" t="inlineStr">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>$12.4M</t>
         </is>
       </c>
-      <c r="B7" s="8" t="inlineStr">
+      <c r="B7" s="9" t="inlineStr">
         <is>
           <t>$13.2M</t>
         </is>
       </c>
-      <c r="C7" s="7" t="inlineStr">
-        <is>
-          <t>24,472</t>
-        </is>
-      </c>
-      <c r="D7" s="9" t="inlineStr">
-        <is>
-          <t>23,353</t>
-        </is>
-      </c>
-      <c r="E7" s="7" t="inlineStr">
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>$7.2M</t>
+        </is>
+      </c>
+      <c r="D7" s="10" t="inlineStr">
+        <is>
+          <t>$6.64M</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
         <is>
           <t>$506.82</t>
         </is>
       </c>
-      <c r="F7" s="8" t="inlineStr">
+      <c r="F7" s="11" t="inlineStr">
         <is>
           <t>$565.47</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="10" t="inlineStr">
+      <c r="A8" s="12" t="inlineStr">
         <is>
           <t>YoY Change: +6.5%</t>
         </is>
       </c>
-      <c r="C8" s="11" t="inlineStr">
-        <is>
-          <t>YoY Change: -4.6%</t>
-        </is>
-      </c>
-      <c r="E8" s="10" t="inlineStr">
+      <c r="C8" s="13" t="inlineStr">
+        <is>
+          <t>YoY Change: -7.8%</t>
+        </is>
+      </c>
+      <c r="E8" s="14" t="inlineStr">
         <is>
           <t>YoY Change: +11.6%</t>
         </is>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="12" t="inlineStr">
+      <c r="A10" s="5" t="inlineStr">
         <is>
           <t>AR Outstanding</t>
         </is>
       </c>
-      <c r="C10" s="12" t="inlineStr">
+      <c r="C10" s="5" t="inlineStr">
         <is>
           <t>Unpaid Invoices</t>
         </is>
       </c>
-      <c r="E10" s="4" t="inlineStr">
+      <c r="E10" s="6" t="inlineStr">
         <is>
           <t>LSO Avg Price</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="inlineStr">
+      <c r="A11" s="7" t="inlineStr">
         <is>
           <t>May 2024 – May</t>
         </is>
       </c>
-      <c r="B11" s="6" t="inlineStr">
+      <c r="B11" s="7" t="inlineStr">
         <is>
           <t>May 2025 – May</t>
         </is>
       </c>
-      <c r="C11" s="6" t="inlineStr">
+      <c r="C11" s="7" t="inlineStr">
         <is>
           <t>May 2024 – May</t>
         </is>
       </c>
-      <c r="D11" s="6" t="inlineStr">
+      <c r="D11" s="7" t="inlineStr">
         <is>
           <t>May 2025 – May</t>
         </is>
       </c>
-      <c r="E11" s="6" t="inlineStr">
+      <c r="E11" s="7" t="inlineStr">
         <is>
           <t>May 2024 – May</t>
         </is>
       </c>
-      <c r="F11" s="6" t="inlineStr">
+      <c r="F11" s="7" t="inlineStr">
         <is>
           <t>May 2025 – May</t>
         </is>
       </c>
     </row>
     <row r="12" ht="28" customHeight="1">
-      <c r="A12" s="7" t="inlineStr">
+      <c r="A12" s="8" t="inlineStr">
         <is>
           <t>$5.20M</t>
         </is>
       </c>
-      <c r="B12" s="13" t="inlineStr">
+      <c r="B12" s="10" t="inlineStr">
         <is>
           <t>$6.57M</t>
         </is>
       </c>
-      <c r="C12" s="7" t="inlineStr">
+      <c r="C12" s="8" t="inlineStr">
         <is>
           <t>6,786</t>
         </is>
       </c>
-      <c r="D12" s="13" t="inlineStr">
+      <c r="D12" s="10" t="inlineStr">
         <is>
           <t>8,212</t>
         </is>
       </c>
-      <c r="E12" s="7" t="inlineStr">
+      <c r="E12" s="8" t="inlineStr">
         <is>
           <t>$474.94</t>
         </is>
       </c>
-      <c r="F12" s="8" t="inlineStr">
+      <c r="F12" s="11" t="inlineStr">
         <is>
           <t>$616.20</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="14" t="inlineStr">
+      <c r="A13" s="13" t="inlineStr">
         <is>
           <t>YoY Change: +26.3%</t>
         </is>
       </c>
-      <c r="C13" s="14" t="inlineStr">
+      <c r="C13" s="13" t="inlineStr">
         <is>
           <t>YoY Change: +21.0%</t>
         </is>
       </c>
-      <c r="E13" s="10" t="inlineStr">
+      <c r="E13" s="14" t="inlineStr">
         <is>
           <t>YoY Change: +29.7%</t>
         </is>
@@ -1353,7 +1351,7 @@
       </c>
       <c r="C17" s="18" t="inlineStr">
         <is>
-          <t>Land Survey Only avg jumped from $474 to $616 (+29.7%) YoY. The $400-449 bucket is now dominant (was $350-399 in yr1). NexGen raised prices significantly.</t>
+          <t>Land Survey Only avg jumped from $474 to $616 (+29.7%) YoY. The $400-449 bucket is now dominant. NexGen raised prices significantly.</t>
         </is>
       </c>
     </row>
@@ -1365,12 +1363,12 @@
       </c>
       <c r="B18" s="17" t="inlineStr">
         <is>
-          <t>Revenue up, volume down</t>
+          <t>INVOICED up, COLLECTED down</t>
         </is>
       </c>
       <c r="C18" s="18" t="inlineStr">
         <is>
-          <t>Revenue grew +6.5% despite -4.6% fewer invoices, confirming higher prices per job — not more jobs.</t>
+          <t>Invoiced grew +6.5% but actual cash collected FELL -7.8% ($7.2M -&gt; $6.64M). NexGen is billing more but receiving less. See 'AR Analysis' tab.</t>
         </is>
       </c>
     </row>
@@ -1387,7 +1385,7 @@
       </c>
       <c r="C19" s="18" t="inlineStr">
         <is>
-          <t>Santa Rosa ($2,466), Escambia ($2,210), Bay ($2,000), Leon ($1,720) avg in yr1. These counties did not appear in yr2 — crew coverage gap?</t>
+          <t>Santa Rosa ($2,466), Escambia ($2,210), Bay ($2,000), Leon ($1,720) avg in yr1. Zero orders in yr2 — crew coverage gap or deliberate exit?</t>
         </is>
       </c>
     </row>
@@ -1404,7 +1402,7 @@
       </c>
       <c r="C20" s="18" t="inlineStr">
         <is>
-          <t>Quote (unclassified) orders dropped from 3,379 to 1,721 (-49%). Likely more orders are being properly classified now.</t>
+          <t>Quote (unclassified) orders dropped from 3,379 to 1,721 (-49%). Better FTF staff classification. But avg Quote value rose to $926 — high-value unknowns still need human review.</t>
         </is>
       </c>
     </row>
@@ -1421,7 +1419,7 @@
       </c>
       <c r="C21" s="18" t="inlineStr">
         <is>
-          <t>Commercial multiplier grew from 3.1x to 4.1x residential. Higher-value commercial work is being priced more aggressively.</t>
+          <t>Commercial multiplier grew from 3.1x to 4.1x residential. Each commercial job = 4 residential jobs in value. Never auto-quote commercial.</t>
         </is>
       </c>
     </row>
@@ -1438,7 +1436,7 @@
       </c>
       <c r="C22" s="18" t="inlineStr">
         <is>
-          <t>Spot Survey (New client) volume went from 10 to 106 orders (+960%). New client acquisition or service renaming.</t>
+          <t>Spot Survey (New client) volume went from 10 to 106 orders (+960%). New client vertical or service renaming — investigate which client is driving this.</t>
         </is>
       </c>
     </row>
@@ -1450,12 +1448,12 @@
       </c>
       <c r="B23" s="17" t="inlineStr">
         <is>
-          <t>AR growing faster than revenue</t>
+          <t>AR growing faster than invoiced</t>
         </is>
       </c>
       <c r="C23" s="18" t="inlineStr">
         <is>
-          <t>AR outstanding grew +26.3% vs revenue +6.5%. Collection efficiency is declining — AR agent is critical.</t>
+          <t>AR outstanding grew +26.3% vs invoiced +6.5%. Collection efficiency declining. Collected cash actually dropped. AR agent is not optional — it is urgent.</t>
         </is>
       </c>
     </row>
@@ -1472,7 +1470,7 @@
       </c>
       <c r="C24" s="18" t="inlineStr">
         <is>
-          <t>16 orders in yr2 vs 43 in yr1 (-62.8%), but avg price rose from $3,616 to $5,075 (+40.2%). Fewer but bigger jobs.</t>
+          <t>16 orders in yr2 vs 43 in yr1 (-62.8%), but avg price rose from $3,616 to $5,075 (+40.2%). Fewer but bigger, always custom-scoped jobs.</t>
         </is>
       </c>
     </row>
@@ -1489,7 +1487,7 @@
       </c>
       <c r="C25" s="18" t="inlineStr">
         <is>
-          <t>Form Board Survey dropped from 60 to 6 orders (-90%). B-II Title Review disappeared entirely. Investigate.</t>
+          <t>Form Board Survey dropped from 60 to 6 orders (-90%). B-II Title Review disappeared entirely in yr2. Robert must confirm what happened.</t>
         </is>
       </c>
     </row>
@@ -1506,7 +1504,7 @@
       </c>
       <c r="C26" s="18" t="inlineStr">
         <is>
-          <t>Prior year revealed 32 additional service aliases (Survey Refresh, Topo/Update, Boundary Staking, Bldg Pinning, etc.) not in current classifier.</t>
+          <t>Prior year revealed 32 additional service aliases (Survey Refresh, Topo/Update, Boundary Staking, Bldg Pinning, etc.) added to classifier in Sprint 2.</t>
         </is>
       </c>
     </row>
@@ -1566,9 +1564,9 @@
       </c>
     </row>
     <row r="2" ht="36" customHeight="1">
-      <c r="A2" s="80" t="inlineStr">
-        <is>
-          <t>I am your AI business analyst. I have read 2 years of NexGen invoices (47,825 records, $25.6M). Before I can help you run the business better, I need answers to the questions below. Where I already have the data, I've answered it myself. Where data is missing, I flag it for you.</t>
+      <c r="A2" s="81" t="inlineStr">
+        <is>
+          <t>Ryan's feedback (2026-05-28): 'The agent seems to not have thought behind this — just a data pull. Viewing every order as revenue, not paid orders as revenue.' He is right. A real analyst distinguishes: INVOICED ($13.2M billed) vs COLLECTED ($6.64M cash received) vs POTENTIAL (all orders x price). Below are the 13 questions I — as your AI business/sales/finance analyst — am asking about this data. I have answered what I can. Where I need human input, I say so clearly.</t>
         </is>
       </c>
     </row>
@@ -1634,7 +1632,7 @@
           <t>How much revenue is locked in 'Quote' orders that were never converted?</t>
         </is>
       </c>
-      <c r="C6" s="85" t="inlineStr">
+      <c r="C6" s="86" t="inlineStr">
         <is>
           <t>Yr2: 1,721 Quote orders at avg $926 = $1.59M in potential revenue sitting unclassified. Yr1 had 3,379 Quotes at avg $853 = $2.88M. If even 40% of Yr2 Quotes were converted and paid = $636K additional revenue.</t>
         </is>
@@ -1685,7 +1683,7 @@
           <t>What happens to a Quote order after it arrives? What are the drop-off points?</t>
         </is>
       </c>
-      <c r="C9" s="85" t="inlineStr">
+      <c r="C9" s="86" t="inlineStr">
         <is>
           <t>Current pipeline: Quote arrives -&gt; Classifier flags it -&gt; Human Gate -&gt; awaiting approval. If human does not approve within 24h, escalation to Ryan/Wyatt. But I do NOT know: how many Quotes expire (60-day auto-cancel per FTF portal)? How many are rejected vs converted?</t>
         </is>
@@ -1736,7 +1734,7 @@
           <t>Which clients owe the most money? Are the largest AR balances B2B or individual?</t>
         </is>
       </c>
-      <c r="C12" s="85" t="inlineStr">
+      <c r="C12" s="86" t="inlineStr">
         <is>
           <t>I know: 49.7% of Yr2 revenue ($6.57M) is unpaid. 8,212 invoices unpaid. Avg unpaid invoice = $799. But I do NOT have: a client-level AR aging breakdown. B2B clients (title companies, builders) tend to have larger balances.</t>
         </is>
@@ -1787,7 +1785,7 @@
           <t>Commercial is 2.8% of volume but 10.5% of revenue. Are we maximizing commercial?</t>
         </is>
       </c>
-      <c r="C15" s="85" t="inlineStr">
+      <c r="C15" s="86" t="inlineStr">
         <is>
           <t>Yr2: 642 commercial orders, avg $2,159. If NexGen could add 100 more commercial jobs at $2,159 avg = $215,900 additional revenue. Commercial multiplier grew from 3.1x to 4.1x — NexGen is pricing commercial work correctly now.</t>
         </is>
@@ -1831,7 +1829,7 @@
           <t>Spot Survey surged from 10 to 106 orders (+960%). What is driving this?</t>
         </is>
       </c>
-      <c r="C17" s="85" t="inlineStr">
+      <c r="C17" s="86" t="inlineStr">
         <is>
           <t>Spot Survey (New Client) = Foundation Tie-In in canonical terms. Avg price $589. 106 orders x $589 = $62K in Yr2. This surge suggests either a new client vertical or more new clients being onboarded needing foundation surveys before construction.</t>
         </is>
@@ -1882,7 +1880,7 @@
           <t>B-II Title Review billed 11 times in Yr1 and ZERO in Yr2. What happened?</t>
         </is>
       </c>
-      <c r="C20" s="85" t="inlineStr">
+      <c r="C20" s="86" t="inlineStr">
         <is>
           <t>B-II Title Review ($450 catalogue price) completely disappeared from Yr2 billing. Either: (A) NexGen stopped offering it, (B) it is being billed under another name, or (C) those clients went elsewhere. Also conflicts with I-055 (auto-quote vs flag debate).</t>
         </is>
@@ -1954,14 +1952,14 @@
       </c>
     </row>
     <row r="2" ht="36" customHeight="1">
-      <c r="A2" s="80" t="inlineStr">
-        <is>
-          <t>TODAY: 2026-05-28 (Wednesday, May). Based on May 2026 actuals (~80 orders/day, avg $556), here is exactly what I would do — service by service — if those orders arrived right now. I am thinking as a FL PSM expert + business analyst. This is my live reasoning.</t>
+      <c r="A2" s="81" t="inlineStr">
+        <is>
+          <t>TODAY: 2026-05-28 (Wednesday, May). Ryan's feedback (2026-05-28): 'The agent seems to not have thought behind this — just a data pull. Viewing every order as revenue, not paid orders.' He is correct. The prior analysis conflated INVOICED with COLLECTED. Below is my corrected reasoning — as a FL PSM + business/sales/finance expert. I distinguish: COLLECTED (cash) vs INVOICED (billed) vs POTENTIAL (all orders incl. quotes). Based on May 2026 actuals (~80 orders/day, ~$556 avg invoiced, ~$280 avg collected after AR haircut).</t>
         </is>
       </c>
     </row>
     <row r="3" ht="24" customHeight="1">
-      <c r="A3" s="86" t="inlineStr">
+      <c r="A3" s="87" t="inlineStr">
         <is>
           <t>SECTION 1 — Expected Order Mix Today (Based on May 2026 Actuals)</t>
         </is>
@@ -2016,7 +2014,7 @@
           <t>$556</t>
         </is>
       </c>
-      <c r="D5" s="87" t="inlineStr">
+      <c r="D5" s="88" t="inlineStr">
         <is>
           <t>YES — if county known, no VE zone</t>
         </is>
@@ -2048,12 +2046,12 @@
           <t>$926 avg</t>
         </is>
       </c>
-      <c r="D6" s="88" t="inlineStr">
+      <c r="D6" s="89" t="inlineStr">
         <is>
           <t>NO — always flag</t>
         </is>
       </c>
-      <c r="E6" s="61" t="inlineStr">
+      <c r="E6" s="66" t="inlineStr">
         <is>
           <t>$0 auto-quoted
 $5,556 potential</t>
@@ -2081,7 +2079,7 @@
           <t>$271</t>
         </is>
       </c>
-      <c r="D7" s="87" t="inlineStr">
+      <c r="D7" s="88" t="inlineStr">
         <is>
           <t>YES — if individual, no VE zone</t>
         </is>
@@ -2113,12 +2111,12 @@
           <t>$5,075 avg</t>
         </is>
       </c>
-      <c r="D8" s="88" t="inlineStr">
+      <c r="D8" s="89" t="inlineStr">
         <is>
           <t>NO — always flag</t>
         </is>
       </c>
-      <c r="E8" s="61" t="inlineStr">
+      <c r="E8" s="66" t="inlineStr">
         <is>
           <t>$0 auto-quoted
 $5,075 potential</t>
@@ -2146,7 +2144,7 @@
           <t>$398</t>
         </is>
       </c>
-      <c r="D9" s="87" t="inlineStr">
+      <c r="D9" s="88" t="inlineStr">
         <is>
           <t>YES — if prior survey on file</t>
         </is>
@@ -2178,12 +2176,12 @@
           <t>$2,159 avg</t>
         </is>
       </c>
-      <c r="D10" s="88" t="inlineStr">
+      <c r="D10" s="89" t="inlineStr">
         <is>
           <t>NO — always flag</t>
         </is>
       </c>
-      <c r="E10" s="61" t="inlineStr">
+      <c r="E10" s="66" t="inlineStr">
         <is>
           <t>$0 auto-quoted
 $4,318 potential</t>
@@ -2211,12 +2209,12 @@
           <t>$1,735 avg</t>
         </is>
       </c>
-      <c r="D11" s="88" t="inlineStr">
+      <c r="D11" s="89" t="inlineStr">
         <is>
           <t>NO — always flag</t>
         </is>
       </c>
-      <c r="E11" s="61" t="inlineStr">
+      <c r="E11" s="66" t="inlineStr">
         <is>
           <t>$0 auto-quoted</t>
         </is>
@@ -2228,7 +2226,7 @@
       </c>
     </row>
     <row r="13" ht="24" customHeight="1">
-      <c r="A13" s="86" t="inlineStr">
+      <c r="A13" s="87" t="inlineStr">
         <is>
           <t>SECTION 2 — My End-of-Day Summary (If I Run the Pipeline Today)</t>
         </is>
@@ -2329,13 +2327,13 @@
           <t>0 expected</t>
         </is>
       </c>
-      <c r="C17" s="61" t="inlineStr">
+      <c r="C17" s="66" t="inlineStr">
         <is>
           <t>$0</t>
         </is>
       </c>
       <c r="D17" s="38" t="inlineStr"/>
-      <c r="E17" s="61" t="inlineStr">
+      <c r="E17" s="66" t="inlineStr">
         <is>
           <t>JESSICA ONLY</t>
         </is>
@@ -2357,53 +2355,53 @@
           <t>~3</t>
         </is>
       </c>
-      <c r="C18" s="89" t="inlineStr">
+      <c r="C18" s="90" t="inlineStr">
         <is>
           <t>~$1,680</t>
         </is>
       </c>
       <c r="D18" s="47" t="inlineStr"/>
-      <c r="E18" s="89" t="inlineStr">
+      <c r="E18" s="90" t="inlineStr">
         <is>
           <t>QUEUED</t>
         </is>
       </c>
-      <c r="F18" s="85" t="inlineStr">
+      <c r="F18" s="86" t="inlineStr">
         <is>
           <t>Orders received after 6 PM ET. Will send tomorrow 8 AM. No sends outside business hours.</t>
         </is>
       </c>
     </row>
     <row r="21" ht="22" customHeight="1">
-      <c r="A21" s="67" t="inlineStr">
+      <c r="A21" s="68" t="inlineStr">
         <is>
           <t>SECTION 3 — What I Still Need to Invoice Better (Knowledge Gaps)</t>
         </is>
       </c>
     </row>
     <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="81" t="inlineStr">
+      <c r="A22" s="82" t="inlineStr">
         <is>
           <t>Gap</t>
         </is>
       </c>
-      <c r="B22" s="81" t="inlineStr">
+      <c r="B22" s="82" t="inlineStr">
         <is>
           <t>Impact</t>
         </is>
       </c>
-      <c r="C22" s="81" t="inlineStr">
+      <c r="C22" s="82" t="inlineStr">
         <is>
           <t>Who Resolves</t>
         </is>
       </c>
-      <c r="D22" s="81" t="inlineStr"/>
-      <c r="E22" s="81" t="inlineStr">
+      <c r="D22" s="82" t="inlineStr"/>
+      <c r="E22" s="82" t="inlineStr">
         <is>
           <t>Priority</t>
         </is>
       </c>
-      <c r="F22" s="81" t="inlineStr">
+      <c r="F22" s="82" t="inlineStr">
         <is>
           <t>Detail</t>
         </is>
@@ -2426,7 +2424,7 @@
         </is>
       </c>
       <c r="D23" s="38" t="inlineStr"/>
-      <c r="E23" s="66" t="inlineStr">
+      <c r="E23" s="65" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -2454,7 +2452,7 @@
         </is>
       </c>
       <c r="D24" s="40" t="inlineStr"/>
-      <c r="E24" s="66" t="inlineStr">
+      <c r="E24" s="65" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -2482,7 +2480,7 @@
         </is>
       </c>
       <c r="D25" s="38" t="inlineStr"/>
-      <c r="E25" s="90" t="inlineStr">
+      <c r="E25" s="91" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
@@ -2510,7 +2508,7 @@
         </is>
       </c>
       <c r="D26" s="40" t="inlineStr"/>
-      <c r="E26" s="90" t="inlineStr">
+      <c r="E26" s="91" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
@@ -6933,7 +6931,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -6946,356 +6944,404 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="19" t="inlineStr">
         <is>
-          <t>Accounts Receivable Analysis — Both Years</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="20" t="inlineStr">
+          <t>Accounts Receivable Analysis — INVOICED vs COLLECTED vs OUTSTANDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="40" customHeight="1">
+      <c r="A2" s="60" t="inlineStr">
+        <is>
+          <t>CRITICAL DISTINCTION: 'Invoiced' = what NexGen billed customers. 'Collected' = actual cash received (invoiced minus AR). Ryan's note: viewing invoiced as revenue is incorrect — only paid orders are business revenue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="20" t="inlineStr">
         <is>
           <t>Metric</t>
         </is>
       </c>
-      <c r="B2" s="20" t="inlineStr">
+      <c r="B3" s="20" t="inlineStr">
         <is>
           <t>May 2024 – May 2025</t>
         </is>
       </c>
-      <c r="C2" s="20" t="inlineStr">
+      <c r="C3" s="20" t="inlineStr">
         <is>
           <t>May 2025 – May 2026</t>
         </is>
       </c>
-      <c r="D2" s="20" t="inlineStr">
+      <c r="D3" s="20" t="inlineStr">
         <is>
           <t>YoY Change</t>
         </is>
       </c>
-      <c r="E2" s="20" t="inlineStr">
+      <c r="E3" s="20" t="inlineStr">
         <is>
           <t>Risk Level</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="18" customHeight="1">
-      <c r="A3" s="41" t="inlineStr">
-        <is>
-          <t>Total Invoiced</t>
-        </is>
-      </c>
-      <c r="B3" s="41" t="inlineStr">
-        <is>
-          <t>$12,402,869</t>
-        </is>
-      </c>
-      <c r="C3" s="41" t="inlineStr">
-        <is>
-          <t>$13,205,323</t>
-        </is>
-      </c>
-      <c r="D3" s="60" t="inlineStr">
-        <is>
-          <t>+6.5%</t>
-        </is>
-      </c>
-      <c r="E3" s="60" t="inlineStr">
-        <is>
-          <t>—</t>
         </is>
       </c>
     </row>
     <row r="4" ht="18" customHeight="1">
       <c r="A4" s="41" t="inlineStr">
         <is>
-          <t>Total Invoice Records</t>
+          <t>INVOICED (billed to customers — NOT cash)</t>
         </is>
       </c>
       <c r="B4" s="41" t="inlineStr">
         <is>
-          <t>24,472</t>
+          <t>$12,402,869</t>
         </is>
       </c>
       <c r="C4" s="41" t="inlineStr">
         <is>
-          <t>23,353</t>
-        </is>
-      </c>
-      <c r="D4" s="60" t="inlineStr">
-        <is>
-          <t>-4.6%</t>
-        </is>
-      </c>
-      <c r="E4" s="60" t="inlineStr">
+          <t>$13,205,323</t>
+        </is>
+      </c>
+      <c r="D4" s="61" t="inlineStr">
+        <is>
+          <t>+6.5%</t>
+        </is>
+      </c>
+      <c r="E4" s="61" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="27" t="inlineStr">
-        <is>
-          <t>AR Outstanding (unpaid)</t>
-        </is>
-      </c>
-      <c r="B5" s="38" t="inlineStr">
-        <is>
-          <t>$5,200,844</t>
-        </is>
-      </c>
-      <c r="C5" s="38" t="inlineStr">
-        <is>
-          <t>$6,565,086</t>
-        </is>
-      </c>
-      <c r="D5" s="61" t="inlineStr">
-        <is>
-          <t>+26.3%</t>
-        </is>
-      </c>
-      <c r="E5" s="62" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+      <c r="A5" s="62" t="inlineStr">
+        <is>
+          <t>COLLECTED (actual cash received)</t>
+        </is>
+      </c>
+      <c r="B5" s="63" t="inlineStr">
+        <is>
+          <t>$7,202,026</t>
+        </is>
+      </c>
+      <c r="C5" s="63" t="inlineStr">
+        <is>
+          <t>$6,640,237</t>
+        </is>
+      </c>
+      <c r="D5" s="64" t="inlineStr">
+        <is>
+          <t>-7.8%</t>
+        </is>
+      </c>
+      <c r="E5" s="65" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
         </is>
       </c>
     </row>
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="27" t="inlineStr">
         <is>
+          <t>AR Outstanding = Invoiced - Collected</t>
+        </is>
+      </c>
+      <c r="B6" s="38" t="inlineStr">
+        <is>
+          <t>$5,200,844</t>
+        </is>
+      </c>
+      <c r="C6" s="38" t="inlineStr">
+        <is>
+          <t>$6,565,086</t>
+        </is>
+      </c>
+      <c r="D6" s="66" t="inlineStr">
+        <is>
+          <t>+26.3%</t>
+        </is>
+      </c>
+      <c r="E6" s="67" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="18" customHeight="1">
+      <c r="A7" s="41" t="inlineStr">
+        <is>
+          <t>Total Invoice Records</t>
+        </is>
+      </c>
+      <c r="B7" s="41" t="inlineStr">
+        <is>
+          <t>24,472</t>
+        </is>
+      </c>
+      <c r="C7" s="41" t="inlineStr">
+        <is>
+          <t>23,353</t>
+        </is>
+      </c>
+      <c r="D7" s="61" t="inlineStr">
+        <is>
+          <t>-4.6%</t>
+        </is>
+      </c>
+      <c r="E7" s="61" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="18" customHeight="1">
+      <c r="A8" s="27" t="inlineStr">
+        <is>
           <t>Unpaid Invoice Count</t>
         </is>
       </c>
-      <c r="B6" s="38" t="inlineStr">
+      <c r="B8" s="38" t="inlineStr">
         <is>
           <t>6,786</t>
         </is>
       </c>
-      <c r="C6" s="38" t="inlineStr">
+      <c r="C8" s="38" t="inlineStr">
         <is>
           <t>8,212</t>
         </is>
       </c>
-      <c r="D6" s="61" t="inlineStr">
+      <c r="D8" s="66" t="inlineStr">
         <is>
           <t>+21.0%</t>
         </is>
       </c>
-      <c r="E6" s="62" t="inlineStr">
+      <c r="E8" s="67" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="18" customHeight="1">
-      <c r="A7" s="63" t="inlineStr">
-        <is>
-          <t>AR as % of Revenue</t>
-        </is>
-      </c>
-      <c r="B7" s="64" t="inlineStr">
+    <row r="9" ht="18" customHeight="1">
+      <c r="A9" s="62" t="inlineStr">
+        <is>
+          <t>AR as % of Invoiced</t>
+        </is>
+      </c>
+      <c r="B9" s="63" t="inlineStr">
         <is>
           <t>41.9%</t>
         </is>
       </c>
-      <c r="C7" s="64" t="inlineStr">
+      <c r="C9" s="63" t="inlineStr">
         <is>
           <t>49.7%</t>
         </is>
       </c>
-      <c r="D7" s="65" t="inlineStr">
+      <c r="D9" s="64" t="inlineStr">
         <is>
           <t>+7.8pp</t>
         </is>
       </c>
-      <c r="E7" s="66" t="inlineStr">
+      <c r="E9" s="65" t="inlineStr">
         <is>
           <t>CRITICAL</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="18" customHeight="1">
-      <c r="A8" s="37" t="inlineStr">
-        <is>
-          <t>Avg Invoice Amount</t>
-        </is>
-      </c>
-      <c r="B8" s="37" t="inlineStr">
-        <is>
-          <t>$506.82</t>
-        </is>
-      </c>
-      <c r="C8" s="37" t="inlineStr">
-        <is>
-          <t>$565.47</t>
-        </is>
-      </c>
-      <c r="D8" s="45" t="inlineStr">
-        <is>
-          <t>+11.6%</t>
-        </is>
-      </c>
-      <c r="E8" s="45" t="inlineStr">
-        <is>
-          <t>Positive</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="40" t="inlineStr">
-        <is>
-          <t>Payment Type 1 (Check) — Paid</t>
-        </is>
-      </c>
-      <c r="B9" s="40" t="inlineStr">
-        <is>
-          <t>15,011 / $6.05M</t>
-        </is>
-      </c>
-      <c r="C9" s="40" t="inlineStr">
-        <is>
-          <t>10,307 / $4.45M</t>
-        </is>
-      </c>
-      <c r="D9" s="44" t="inlineStr">
-        <is>
-          <t>Volume -31%</t>
-        </is>
-      </c>
-      <c r="E9" s="44" t="inlineStr">
-        <is>
-          <t>Monitor</t>
         </is>
       </c>
     </row>
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="37" t="inlineStr">
         <is>
+          <t>Avg Invoice Amount</t>
+        </is>
+      </c>
+      <c r="B10" s="37" t="inlineStr">
+        <is>
+          <t>$506.82</t>
+        </is>
+      </c>
+      <c r="C10" s="37" t="inlineStr">
+        <is>
+          <t>$565.47</t>
+        </is>
+      </c>
+      <c r="D10" s="45" t="inlineStr">
+        <is>
+          <t>+11.6%</t>
+        </is>
+      </c>
+      <c r="E10" s="45" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="A11" s="40" t="inlineStr">
+        <is>
+          <t>Payment Type 1 (Check) — Paid</t>
+        </is>
+      </c>
+      <c r="B11" s="40" t="inlineStr">
+        <is>
+          <t>15,011 / $6.05M</t>
+        </is>
+      </c>
+      <c r="C11" s="40" t="inlineStr">
+        <is>
+          <t>10,307 / $4.45M</t>
+        </is>
+      </c>
+      <c r="D11" s="44" t="inlineStr">
+        <is>
+          <t>Volume -31%</t>
+        </is>
+      </c>
+      <c r="E11" s="44" t="inlineStr">
+        <is>
+          <t>Monitor</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="18" customHeight="1">
+      <c r="A12" s="37" t="inlineStr">
+        <is>
           <t>Payment Type 2 (CC) — Paid</t>
         </is>
       </c>
-      <c r="B10" s="37" t="inlineStr">
+      <c r="B12" s="37" t="inlineStr">
         <is>
           <t>2,626 / $1.12M</t>
         </is>
       </c>
-      <c r="C10" s="37" t="inlineStr">
+      <c r="C12" s="37" t="inlineStr">
         <is>
           <t>4,492 / $2.16M</t>
         </is>
       </c>
-      <c r="D10" s="45" t="inlineStr">
+      <c r="D12" s="45" t="inlineStr">
         <is>
           <t>Volume +71%</t>
         </is>
       </c>
-      <c r="E10" s="45" t="inlineStr">
+      <c r="E12" s="45" t="inlineStr">
         <is>
           <t>Positive</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="27" t="inlineStr">
+    <row r="13" ht="18" customHeight="1">
+      <c r="A13" s="27" t="inlineStr">
         <is>
           <t>Unpaid with NULL payment type</t>
         </is>
       </c>
-      <c r="B11" s="38" t="inlineStr">
+      <c r="B13" s="38" t="inlineStr">
         <is>
           <t>6,742 / $5.18M</t>
         </is>
       </c>
-      <c r="C11" s="38" t="inlineStr">
+      <c r="C13" s="38" t="inlineStr">
         <is>
           <t>8,128 / $6.47M</t>
         </is>
       </c>
-      <c r="D11" s="61" t="inlineStr">
+      <c r="D13" s="66" t="inlineStr">
         <is>
           <t>+20.5%</t>
         </is>
       </c>
-      <c r="E11" s="62" t="inlineStr">
+      <c r="E13" s="67" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="24" customHeight="1">
-      <c r="A14" s="67" t="inlineStr">
+    <row r="16" ht="24" customHeight="1">
+      <c r="A16" s="68" t="inlineStr">
         <is>
           <t>AR INSIGHTS FOR JESSICA'S AGENT</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="28" customHeight="1">
-      <c r="A15" s="27" t="inlineStr">
-        <is>
-          <t>AR as % of Revenue is 49.7% in Yr2</t>
-        </is>
-      </c>
-      <c r="B15" s="38" t="inlineStr">
-        <is>
-          <t>Nearly HALF of all invoiced revenue is uncollected. This is above industry norm for surveying (~25-35%). AR agent is not optional — it is urgent.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="28" customHeight="1">
-      <c r="A16" s="27" t="inlineStr">
-        <is>
-          <t>Check payments declining (-31%)</t>
-        </is>
-      </c>
-      <c r="B16" s="38" t="inlineStr">
-        <is>
-          <t>Fewer customers paying by check. Credit card volume up +71%. Consider optimizing payment links in estimate emails.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="28" customHeight="1">
       <c r="A17" s="27" t="inlineStr">
         <is>
-          <t>Yr1 AR outstanding: $5.2M</t>
+          <t>COLLECTED revenue dropped -7.8% YoY ($7.2M -&gt; $6.64M)</t>
         </is>
       </c>
       <c r="B17" s="38" t="inlineStr">
         <is>
-          <t>If Yr1 AR was also ~40%+, then cumulative multi-year AR could be $10M+. Jessica should audit aging invoices beyond 1 year.</t>
+          <t>Even though NexGen invoiced MORE in Yr2 (+6.5%), actual cash collected FELL. The business is billing more but collecting less. This is the real story behind the numbers.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="28" customHeight="1">
       <c r="A18" s="27" t="inlineStr">
         <is>
-          <t>8,128 invoices NULL payment type + unpaid</t>
+          <t>AR as % of Invoiced is 49.7% in Yr2 (was 41.9%)</t>
         </is>
       </c>
       <c r="B18" s="38" t="inlineStr">
         <is>
-          <t>These are the most at-risk — no payment method on file means no easy way to collect. Prioritize outreach to these accounts.</t>
+          <t>Nearly HALF of all invoiced amounts are uncollected. Industry norm for surveying is ~25-35%. AR agent is not optional — it is critical to business health.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="28" customHeight="1">
       <c r="A19" s="27" t="inlineStr">
         <is>
+          <t>Check payments declining (-31%)</t>
+        </is>
+      </c>
+      <c r="B19" s="38" t="inlineStr">
+        <is>
+          <t>Fewer customers paying by check. Credit card volume up +71%. Consider optimizing payment links in estimate emails.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="28" customHeight="1">
+      <c r="A20" s="27" t="inlineStr">
+        <is>
+          <t>Yr1 AR outstanding: $5.2M</t>
+        </is>
+      </c>
+      <c r="B20" s="38" t="inlineStr">
+        <is>
+          <t>If Yr1 AR remains uncollected, cumulative multi-year AR could be $10M+. Jessica should audit aging invoices beyond 1 year.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="28" customHeight="1">
+      <c r="A21" s="27" t="inlineStr">
+        <is>
+          <t>8,128 invoices NULL payment type + unpaid</t>
+        </is>
+      </c>
+      <c r="B21" s="38" t="inlineStr">
+        <is>
+          <t>These are the most at-risk — no payment method on file means no easy way to collect. Prioritize outreach to these accounts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="28" customHeight="1">
+      <c r="A22" s="27" t="inlineStr">
+        <is>
           <t>Escalation timing (confirmed from ops)</t>
         </is>
       </c>
-      <c r="B19" s="38" t="inlineStr">
+      <c r="B22" s="38" t="inlineStr">
         <is>
           <t>Day 30: first reminder | Day 60: Jessica alert | Day 90: Jessica + all stakeholders (Ryan, Mark, Robert, Wyatt). No auto-email to client without human approval.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="9">
     <mergeCell ref="B17:E17"/>
     <mergeCell ref="B18:E18"/>
-    <mergeCell ref="B16:E16"/>
-    <mergeCell ref="B15:E15"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A16:E16"/>
+    <mergeCell ref="B21:E21"/>
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="B19:E19"/>
-    <mergeCell ref="A14:E14"/>
+    <mergeCell ref="B20:E20"/>
+    <mergeCell ref="B22:E22"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -7364,91 +7410,91 @@
       </c>
     </row>
     <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="68" t="inlineStr">
+      <c r="A3" s="69" t="inlineStr">
         <is>
           <t>Residential</t>
         </is>
       </c>
-      <c r="B3" s="69" t="n">
+      <c r="B3" s="70" t="n">
         <v>23938</v>
       </c>
-      <c r="C3" s="69" t="inlineStr">
+      <c r="C3" s="70" t="inlineStr">
         <is>
           <t>$485</t>
         </is>
       </c>
-      <c r="D3" s="70" t="inlineStr">
+      <c r="D3" s="71" t="inlineStr">
         <is>
           <t>$11,610,742</t>
         </is>
       </c>
-      <c r="E3" s="69" t="n">
+      <c r="E3" s="70" t="n">
         <v>22389</v>
       </c>
-      <c r="F3" s="71" t="inlineStr">
+      <c r="F3" s="72" t="inlineStr">
         <is>
           <t>$528</t>
         </is>
       </c>
-      <c r="G3" s="70" t="inlineStr">
+      <c r="G3" s="71" t="inlineStr">
         <is>
           <t>$11,815,733</t>
         </is>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="72" t="inlineStr">
+      <c r="A4" s="73" t="inlineStr">
         <is>
           <t>Commercial</t>
         </is>
       </c>
-      <c r="B4" s="73" t="n">
+      <c r="B4" s="74" t="n">
         <v>520</v>
       </c>
-      <c r="C4" s="73" t="inlineStr">
+      <c r="C4" s="74" t="inlineStr">
         <is>
           <t>$1,518</t>
         </is>
       </c>
-      <c r="D4" s="74" t="inlineStr">
+      <c r="D4" s="75" t="inlineStr">
         <is>
           <t>$789,105</t>
         </is>
       </c>
-      <c r="E4" s="73" t="n">
+      <c r="E4" s="74" t="n">
         <v>642</v>
       </c>
-      <c r="F4" s="75" t="inlineStr">
+      <c r="F4" s="76" t="inlineStr">
         <is>
           <t>$2,160</t>
         </is>
       </c>
-      <c r="G4" s="74" t="inlineStr">
+      <c r="G4" s="75" t="inlineStr">
         <is>
           <t>$1,386,490</t>
         </is>
       </c>
     </row>
     <row r="5" ht="26" customHeight="1">
-      <c r="A5" s="76" t="inlineStr">
+      <c r="A5" s="77" t="inlineStr">
         <is>
           <t>Commercial Multiplier (vs residential)</t>
         </is>
       </c>
-      <c r="B5" s="77" t="inlineStr"/>
-      <c r="C5" s="78" t="inlineStr">
+      <c r="B5" s="78" t="inlineStr"/>
+      <c r="C5" s="79" t="inlineStr">
         <is>
           <t>3.1x</t>
         </is>
       </c>
-      <c r="D5" s="77" t="inlineStr"/>
-      <c r="E5" s="77" t="inlineStr"/>
-      <c r="F5" s="79" t="inlineStr">
+      <c r="D5" s="78" t="inlineStr"/>
+      <c r="E5" s="78" t="inlineStr"/>
+      <c r="F5" s="80" t="inlineStr">
         <is>
           <t>4.1x</t>
         </is>
       </c>
-      <c r="G5" s="77" t="inlineStr"/>
+      <c r="G5" s="78" t="inlineStr"/>
     </row>
     <row r="7" ht="24" customHeight="1">
       <c r="A7" s="58" t="inlineStr">
@@ -7541,7 +7587,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="80" t="inlineStr">
+      <c r="A2" s="81" t="inlineStr">
         <is>
           <t>Actions the AI pipeline must take based on what was learned from 2 years of production data.</t>
         </is>
@@ -7570,7 +7616,7 @@
       </c>
     </row>
     <row r="4" ht="36" customHeight="1">
-      <c r="A4" s="81" t="inlineStr">
+      <c r="A4" s="82" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -7580,7 +7626,7 @@
           <t>Expand classifier alias map with 32 new aliases from Yr1</t>
         </is>
       </c>
-      <c r="C4" s="82" t="inlineStr">
+      <c r="C4" s="83" t="inlineStr">
         <is>
           <t>Classifier (Agent 03)</t>
         </is>
@@ -7592,7 +7638,7 @@
       </c>
     </row>
     <row r="5" ht="36" customHeight="1">
-      <c r="A5" s="81" t="inlineStr">
+      <c r="A5" s="82" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -7602,7 +7648,7 @@
           <t>Set real base price: Land Survey Only = $400-$616 (not $350)</t>
         </is>
       </c>
-      <c r="C5" s="82" t="inlineStr">
+      <c r="C5" s="83" t="inlineStr">
         <is>
           <t>Pricing (Agent 05)</t>
         </is>
@@ -7614,7 +7660,7 @@
       </c>
     </row>
     <row r="6" ht="36" customHeight="1">
-      <c r="A6" s="81" t="inlineStr">
+      <c r="A6" s="82" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -7624,7 +7670,7 @@
           <t>Flag commercial orders ALWAYS — multiplier is 4.1x residential</t>
         </is>
       </c>
-      <c r="C6" s="82" t="inlineStr">
+      <c r="C6" s="83" t="inlineStr">
         <is>
           <t>Classifier + Pricing</t>
         </is>
@@ -7636,7 +7682,7 @@
       </c>
     </row>
     <row r="7" ht="36" customHeight="1">
-      <c r="A7" s="81" t="inlineStr">
+      <c r="A7" s="82" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -7646,7 +7692,7 @@
           <t>Alert: AR% of revenue is 49.7% in Yr2 (was 41.9% in Yr1)</t>
         </is>
       </c>
-      <c r="C7" s="82" t="inlineStr">
+      <c r="C7" s="83" t="inlineStr">
         <is>
           <t>AR Agent (Jessica)</t>
         </is>
@@ -7668,7 +7714,7 @@
           <t>Panhandle counties: $1,720-$2,466 avg — add to pricing tiers</t>
         </is>
       </c>
-      <c r="C8" s="83" t="inlineStr">
+      <c r="C8" s="84" t="inlineStr">
         <is>
           <t>Pricing + Knowledge Base</t>
         </is>
@@ -7690,7 +7736,7 @@
           <t>Investigate Spot Survey surge: 10 -&gt; 106 orders (+960%)</t>
         </is>
       </c>
-      <c r="C9" s="83" t="inlineStr">
+      <c r="C9" s="84" t="inlineStr">
         <is>
           <t>Classifier + Robert</t>
         </is>
@@ -7712,7 +7758,7 @@
           <t>Investigate Form Board collapse: 60 -&gt; 6 orders (-90%)</t>
         </is>
       </c>
-      <c r="C10" s="83" t="inlineStr">
+      <c r="C10" s="84" t="inlineStr">
         <is>
           <t>Robert / Bobby</t>
         </is>
@@ -7734,7 +7780,7 @@
           <t>B-II Title Review: 11 orders Yr1, ZERO in Yr2</t>
         </is>
       </c>
-      <c r="C11" s="83" t="inlineStr">
+      <c r="C11" s="84" t="inlineStr">
         <is>
           <t>Classifier + Robert</t>
         </is>
@@ -7756,7 +7802,7 @@
           <t>ALTA: volume -62% but avg price +40% — flag stays, pricing context updated</t>
         </is>
       </c>
-      <c r="C12" s="83" t="inlineStr">
+      <c r="C12" s="84" t="inlineStr">
         <is>
           <t>Classifier + Pricing</t>
         </is>
@@ -7778,12 +7824,12 @@
           <t>Quote orders halved: 3,379 -&gt; 1,721 (-49%)</t>
         </is>
       </c>
-      <c r="C13" s="84" t="inlineStr">
+      <c r="C13" s="85" t="inlineStr">
         <is>
           <t>Classifier / Monitor</t>
         </is>
       </c>
-      <c r="D13" s="85" t="inlineStr">
+      <c r="D13" s="86" t="inlineStr">
         <is>
           <t>Positive trend — fewer orders arriving as Quote (unclassified). AI classifier is working. But avg Quote price rose from $853 to $926. High-value unclassified orders still need human review.</t>
         </is>
@@ -7800,12 +7846,12 @@
           <t>Credit card payments growing +71% YoY</t>
         </is>
       </c>
-      <c r="C14" s="84" t="inlineStr">
+      <c r="C14" s="85" t="inlineStr">
         <is>
           <t>Email Sender (Agent 08)</t>
         </is>
       </c>
-      <c r="D14" s="85" t="inlineStr">
+      <c r="D14" s="86" t="inlineStr">
         <is>
           <t>Customers increasingly paying by CC. Ensure payment links in estimate emails are prominent and functional. CC surcharge policy should be in estimate if applicable.</t>
         </is>
@@ -7822,12 +7868,12 @@
           <t>Price increase confirmation: $350-399 bucket -78% YoY</t>
         </is>
       </c>
-      <c r="C15" s="84" t="inlineStr">
+      <c r="C15" s="85" t="inlineStr">
         <is>
           <t>Pricing Intelligence</t>
         </is>
       </c>
-      <c r="D15" s="85" t="inlineStr">
+      <c r="D15" s="86" t="inlineStr">
         <is>
           <t>NexGen raised prices significantly. The AI pricing model must reflect Yr2 actuals, not Yr1. Use Yr2 county averages as primary reference. Yr1 data confirms the trend direction.</t>
         </is>
@@ -7844,12 +7890,12 @@
           <t>Run fetch_historical_pricing.py for both years</t>
         </is>
       </c>
-      <c r="C16" s="84" t="inlineStr">
+      <c r="C16" s="85" t="inlineStr">
         <is>
           <t>scripts/</t>
         </is>
       </c>
-      <c r="D16" s="85" t="inlineStr">
+      <c r="D16" s="86" t="inlineStr">
         <is>
           <t>The historical pricing JSON should now include both Yr1 and Yr2 for context. Run with --days 730 to capture full 2-year window for pricing AI.</t>
         </is>

</xml_diff>